<commit_message>
Aplicação do Modelo Multivariado
Aplicação do modelo multivariado. O resultado válido é o último arquivo com o final 4.
</commit_message>
<xml_diff>
--- a/06_Roteiros_Estatis/Acompanhamento_Analises_PIBICEM.xlsx
+++ b/06_Roteiros_Estatis/Acompanhamento_Analises_PIBICEM.xlsx
@@ -7,19 +7,20 @@
     <sheet state="visible" name="2_Acompanhamento_Analises" sheetId="2" r:id="rId5"/>
     <sheet state="visible" name="Análises Descritivas" sheetId="3" r:id="rId6"/>
     <sheet state="visible" name="Resumo_Testes" sheetId="4" r:id="rId7"/>
+    <sheet state="visible" name="Source References" sheetId="5" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataChecksum="kVsqiMP93GvFPgFHNvVLCD8HO7TRJCBBfLrJDa3cC2A="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="3tURovucPYpBoxFIIy/dS2d9aPeg/FdaV5N8SOy5Ot4="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="455">
   <si>
     <t>Nível de análise</t>
   </si>
@@ -934,6 +935,21 @@
 2025_12_15_HeatMap_Teste_X_quadrado_regiao_corrigida_X_grande_area_CAPES_ING.png
 2025_12_15_Barras_Teste_X_quadrado_regiao_corrigida_X_grande_area_CAPES.png
 2025_12_15_HeatMap_Teste_X_quadrado_regiao_corrigida_X_grande_area_CAPES.png</t>
+  </si>
+  <si>
+    <t>Análise Inferencial – Modelagem Multivariada</t>
+  </si>
+  <si>
+    <t>Avaliar o efeito independente de características institucionais, regionais e de desempenho acadêmico sobre a intensidade de participação das instituições no PIBIC-EM</t>
+  </si>
+  <si>
+    <t>Modelo Linear Generalizado (GLM) com distribuição Quasi-Poisson e função de ligação log</t>
+  </si>
+  <si>
+    <t>São pesquisadores que, independentemente de estarem no Norte ou no Sul e independentemente do prestígio (IGC) de sua universidade, conseguiram acumular capital científico individual (produtividade) e estão ancorados em categorias administrativas que lhes oferecem condições materiais de sustentar essa atividade a longo prazo. O PIBIC-EM, portanto, não cria novos pesquisadores 'do zero'; ele oferece uma ferramenta de reprodução para aqueles que já estão engajados na lógica da produção científica e possuem suporte institucional para tal.</t>
+  </si>
+  <si>
+    <t>2026_02_10_modelo_multivariado_3_.pdf</t>
   </si>
   <si>
     <t>Quais instituições retornam sistematicamente ao programa?</t>
@@ -1144,106 +1160,400 @@
 2025_12_18_instituicao_com_maior_numero_de_proponentes_centro_oeste.png</t>
   </si>
   <si>
-    <t>1. A Anatomia da Desigualdade</t>
-  </si>
-  <si>
-    <t>Relação Testada</t>
-  </si>
-  <si>
-    <t>Arquivo Ref.</t>
-  </si>
-  <si>
-    <t>Resultado</t>
-  </si>
-  <si>
-    <t>Interpretação para o Artigo</t>
-  </si>
-  <si>
-    <t>Fidelidade x Região x Categoria Adm</t>
-  </si>
-  <si>
-    <t>2025_12_18...Fidelidade...</t>
-  </si>
-  <si>
-    <t>Associação Forte. A chance de ser um pesquisador "Fiel" (alta recorrência) não é aleatória; ela depende drasticamente da combinação entre onde você está e em que tipo de instituição atua.</t>
-  </si>
-  <si>
-    <t>Crucial: O "leaky pipeline" (vazamento) de orientadores é seletivo. Certas regiões/instituições retêm talentos, outras funcionam apenas como portas giratórias (entra e sai).</t>
-  </si>
-  <si>
-    <t>Região x Grande Área</t>
-  </si>
-  <si>
-    <t>2025_12_15...Grande_Area...</t>
-  </si>
-  <si>
-    <t>Associação Significativa. As áreas do conhecimento não se distribuem igualmente no território.</t>
-  </si>
-  <si>
-    <t>O PIBIC-EM não fomenta a ciência de forma neutra; ele reforça vocações regionais preexistentes ou desigualdades de oferta disciplinar.</t>
-  </si>
-  <si>
-    <t>Tipo de IES x IGC</t>
-  </si>
-  <si>
-    <t>2025_12_09...Tipo_IES_x_IGC</t>
-  </si>
-  <si>
-    <t>Fortíssima Associação (Cramer's V alto). Federais quase sempre têm IGC Alto; Privadas variam mais.</t>
-  </si>
-  <si>
-    <t>Justificativa Metodológica: Não podemos colocar "Tipo de IES" e "IGC" no modelo de regressão sem tratar a colinearidade. Elas medem quase a mesma coisa no setor público.</t>
-  </si>
-  <si>
-    <t>Tipo de IES x Região</t>
-  </si>
-  <si>
-    <t>2025_12_09...Tipo_IES_x_Regiao</t>
-  </si>
-  <si>
-    <t>Associação Significativa. O perfil institucional muda conforme a geografia (ex: o Norte depende mais de Federais/Estaduais; o Sul/Sudeste tem mais presença Privada/Comunitária).</t>
-  </si>
-  <si>
-    <t>A política nacional única (café com leite para todos) ignora que a rede institucional de suporte é heterogênea no território.</t>
-  </si>
-  <si>
-    <t>2. A Dinâmica da Recompensa (Achados de Performance)</t>
-  </si>
-  <si>
-    <t>Variável</t>
-  </si>
-  <si>
-    <t>Resultado Atualizado</t>
-  </si>
-  <si>
-    <t>Interpretação Crítica</t>
-  </si>
-  <si>
-    <t>Região</t>
-  </si>
-  <si>
-    <t>Disparidade Confirmada (p &lt; 0.05). Sul (M=2.09) &gt; Norte (M=1.63).</t>
-  </si>
-  <si>
-    <t>O pesquisador do Sul tem uma "sobrevida" maior no programa. O desenho da política favorece a manutenção de vínculos nessa região.</t>
-  </si>
-  <si>
-    <t>Tipo de IES</t>
-  </si>
-  <si>
-    <t>Tendência (p = 0.079). Privadas (M=2.16) &gt; Federais (M=1.77).</t>
-  </si>
-  <si>
-    <t>Apesar da força estrutural das Federais, o pesquisador da Privada que entra tende a ficar mais. Isso sugere que, para a Privada, o PIBIC-EM pode ser uma estratégia institucional vital de captação de recursos, gerando maior pressão por recorrência.</t>
-  </si>
-  <si>
-    <t>Produção ($h-index$)</t>
-  </si>
-  <si>
-    <t>Não Significativo (p = 0.419).</t>
-  </si>
-  <si>
-    <t>O Achado Contra-Intuitivo: A "elite produtiva" não domina a recorrência. O programa é permeável a diferentes perfis produtivos, mas geograficamente excludente.</t>
+    <t>Variáveis e Características</t>
+  </si>
+  <si>
+    <t>Resultados Estatísticos (Média/Frequência/X²)</t>
+  </si>
+  <si>
+    <t>P-valor e Significância</t>
+  </si>
+  <si>
+    <t>Tamanho do Efeito/Associação (Inferred)</t>
+  </si>
+  <si>
+    <t>Interpretação e Conclusões</t>
+  </si>
+  <si>
+    <t>Fonte</t>
+  </si>
+  <si>
+    <t>Macro (Geral)</t>
+  </si>
+  <si>
+    <t>Distribuição nacional e histórica de bolsas de Iniciação Científica (IC e ICJ)</t>
+  </si>
+  <si>
+    <t>Crescimento de 1.321 (1984) para 27.717 (2015) bolsas de IC; ICJ saltou de 2% (2003) para 28% (2015) do total.</t>
+  </si>
+  <si>
+    <t>Not in source</t>
+  </si>
+  <si>
+    <t>Forte tendência de crescimento e valorização histórica.</t>
+  </si>
+  <si>
+    <t>A Iniciação Científica consolidou-se como estratégia central de Estado para identificação precoce de talentos e redução do tempo de titulação na pós-graduação.</t>
+  </si>
+  <si>
+    <t>1-4</t>
+  </si>
+  <si>
+    <t>Macro (Regional)</t>
+  </si>
+  <si>
+    <t>Concentração de programas e bolsas de IC/PIBIC-EM por Região Geográfica</t>
+  </si>
+  <si>
+    <t>Sudeste (40,5% a 63%); Nordeste (26,5%); Norte (15,5%); Centro-Oeste (11%); Sul (6,5% a 39.995 bolsas).</t>
+  </si>
+  <si>
+    <t>Forte desigualdade regional e concentração de recursos.</t>
+  </si>
+  <si>
+    <t>Há uma predominância histórica das regiões Sul e Sudeste, refletindo desigualdades na infraestrutura de pesquisa e a necessidade de políticas de desconcentração para evitar a "migração de cérebros".</t>
+  </si>
+  <si>
+    <t>2-7</t>
+  </si>
+  <si>
+    <t>Institucional</t>
+  </si>
+  <si>
+    <t>Distribuição da amostra por Categoria Administrativa das IES (PIBIC-EM)</t>
+  </si>
+  <si>
+    <t>Federal: 56,2% a 59,9%; Privada: 20,5% a 21,9%; Estadual: 14,8% a 15,4%; Municipal/Outras: 2,8% a 3,1%.</t>
+  </si>
+  <si>
+    <t>Predomínio absoluto do setor público federal.</t>
+  </si>
+  <si>
+    <t>O programa PIBIC-EM é majoritariamente executado e ancorado em universidades federais, que atuam como eixo estruturante da pesquisa científica nacional.</t>
+  </si>
+  <si>
+    <t>8-10</t>
+  </si>
+  <si>
+    <t>Institucional (Qualidade)</t>
+  </si>
+  <si>
+    <t>Associação entre Tipo de Instituição (IES) e Índice Geral de Cursos (IGC)</t>
+  </si>
+  <si>
+    <t>$X^2(3) = 30,0$  e  $X^2(8) = 482$ . Universidades Federais detêm entre 84,5% e 98,4% do grupo IGC Alto.</t>
+  </si>
+  <si>
+    <t>$p &lt; 0,001$  (Altamente significativo)</t>
+  </si>
+  <si>
+    <t>V de Cramer = 0,243 a 0,667 (Moderado a Muito Forte).</t>
+  </si>
+  <si>
+    <t>Observa-se uma concentração maciça de indicadores de alta qualidade (IGC Alto) em instituições federais, enquanto privadas e municipais associam-se ao IGC Médio.</t>
+  </si>
+  <si>
+    <t>8, 11-15</t>
+  </si>
+  <si>
+    <t>Regional (Diferenciação)</t>
+  </si>
+  <si>
+    <t>Associação entre Categoria Administrativa da IES e Região Geográfica</t>
+  </si>
+  <si>
+    <t>$X^2(16) = 93,4$  e  $X^2(32) = 126$ .</t>
+  </si>
+  <si>
+    <t>V de Cramer = 0,208 a 0,241 (Moderado).</t>
+  </si>
+  <si>
+    <t>Federais são cruciais para a interiorização no Norte/Nordeste; IES privadas concentram-se no Sul/Sudeste. O Sul apresenta super-representação de IES com IGC Alto.</t>
+  </si>
+  <si>
+    <t>12, 16, 17</t>
+  </si>
+  <si>
+    <t>Grande Área</t>
+  </si>
+  <si>
+    <t>Participação e médias de chamadas do PIBIC-EM por Grande Área (CAPES)</t>
+  </si>
+  <si>
+    <t>Engenharias ( $M=2,67$ ); Saúde ( $M=1,96$ ); Biológicas/Exatas ( $M=1,92$ ); Humanas ( $M=1,77$ ). ANOVA:  $F(8, 26,6) = 1,30$ .</t>
+  </si>
+  <si>
+    <t>$p = 0,286$  (Não significativo)</t>
+  </si>
+  <si>
+    <t>$\epsilon^2 = 0,0144$  (Efeito desprezível).</t>
+  </si>
+  <si>
+    <t>A adesão ao programa é homogênea entre as grandes áreas; as diferenças nas médias são explicadas por trajetórias individuais e não por padrões sistêmicos das áreas.</t>
+  </si>
+  <si>
+    <t>8, 18-21</t>
+  </si>
+  <si>
+    <t>Específico (Associação)</t>
+  </si>
+  <si>
+    <t>Associação entre Tipo de IES e Nível de Produção Acadêmica</t>
+  </si>
+  <si>
+    <t>$X^2(8) = 35,1$ .</t>
+  </si>
+  <si>
+    <t>$p &lt; 0,001$  (Significativo)</t>
+  </si>
+  <si>
+    <t>V de Cramer = 0,180 (Pequeno a moderado).</t>
+  </si>
+  <si>
+    <t>Instituições públicas estaduais e institutos de pesquisa tendem a apresentar alta produção; Federais mostram perfil de produção média/baixa na amostra específica.</t>
+  </si>
+  <si>
+    <t>8, 9</t>
+  </si>
+  <si>
+    <t>Específico (Recorrência)</t>
+  </si>
+  <si>
+    <t>Diferença no número de chamadas participadas por Tipo de IES e IGC</t>
+  </si>
+  <si>
+    <t>Média Privada ( $M=2,16$ ) vs Federal ( $M=1,77$ ); IGC Alto ( $M=1,87$ ) vs Médio ( $M=1,86$ ). Welch's  $F = 2,19$ .</t>
+  </si>
+  <si>
+    <t>$p = 0,079$  e  $p = 0,477$  (Não significativo)</t>
+  </si>
+  <si>
+    <t>$r_{rb} = -0,04$  (Inexpressivo).</t>
+  </si>
+  <si>
+    <t>O tipo de gestão institucional ou o nível do IGC não determinam a intensidade de participação (recorrência) do pesquisador no programa.</t>
+  </si>
+  <si>
+    <t>8, 9, 22-26</t>
+  </si>
+  <si>
+    <t>Colinearidade entre Tipo de IES e Natureza Jurídica/Administrativa</t>
+  </si>
+  <si>
+    <t>$X^2(28) = 2164$ .</t>
+  </si>
+  <si>
+    <t>$p &lt; 0,001$  (Significância total)</t>
+  </si>
+  <si>
+    <t>Coeficiente de Contingência = 0,894 (Extremamente alto).</t>
+  </si>
+  <si>
+    <t>Existe uma colinearidade rígida; cada tipo de instituição está estritamente vinculado à sua natureza jurídica, sem casos híbridos significativos.</t>
+  </si>
+  <si>
+    <t>12, 27</t>
+  </si>
+  <si>
+    <t>Validação Estatística</t>
+  </si>
+  <si>
+    <t>Testes de Normalidade e Homogeneidade (Resíduos das Chamadas)</t>
+  </si>
+  <si>
+    <t>Shapiro-Wilk:  $W=0,811$ ; Levene:  $F(8,532)=0,96$ .</t>
+  </si>
+  <si>
+    <t>$W: p &lt; 0,001$ ;  $F: p=0,469$ .</t>
+  </si>
+  <si>
+    <t>Violação da normalidade; homogeneidade preservada.</t>
+  </si>
+  <si>
+    <t>A variância é homogênea, mas a violação da normalidade sugere que a distribuição de bolsas não segue um padrão normal puro, exigindo cautela na ANOVA.</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>Evolução Econômica</t>
+  </si>
+  <si>
+    <t>Correlação entre valor das bolsas, salário mínimo e inflação (1996-2015)</t>
+  </si>
+  <si>
+    <t>1996: 4,77 salários; 2015: 3,02 salários. Inflação acumulada: 122,95%.</t>
+  </si>
+  <si>
+    <t>Redução acentuada (Depreciação) do poder de compra.</t>
+  </si>
+  <si>
+    <t>O investimento real diminuiu; a bolsa equivale a cerca de 40% do salário mínimo, o que pode desestimular a entrada de jovens de baixa renda.</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>Gestão e Política</t>
+  </si>
+  <si>
+    <t>Execução de metas e fomento (PIBIC-EM/PIBIC-Jr)</t>
+  </si>
+  <si>
+    <t>Crescimento de 377 (2003) para 4.053 (2010) bolsas PIBIC-Jr.</t>
+  </si>
+  <si>
+    <t>Crescimento superior a 1.000%.</t>
+  </si>
+  <si>
+    <t>Consolidação da política de formação inicial, embora haja hiatos entre a formulação estratégica e a implementação tático-operacional no CNPq.</t>
+  </si>
+  <si>
+    <t>3, 28</t>
+  </si>
+  <si>
+    <t>Index</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Iniciação Científica Júnior desafios à materialização de um círculo virtuoso.pdf</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>A História e os objetivos da Iniciação Científica no Ensino Médio uma análise a partir dos programas do Estado do Rio de Janeiro.pdf</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>A iniciação à pesquisa no Brasil políticas de formação de jovens pesquisadores.pdf</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>A_iniciacao_a_pesquisa_no_Brasil_politicas_de_form.pdf</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>Programas de iniciação científica para o ensino médio no Brasil.pdf</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>A iniciação científica no contexto da Educação Básica - Um estudo Baseado na Analálise da Produção Acadêmica.docx</t>
+  </si>
+  <si>
+    <t>iniciacao-cientifica-junior-as-politicas-publicas-de-fomento-a-formacao-de-pesquisadores-na-educacao-basica-brasileira.pdf</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>2025_11_20_participacao_PIBIC-EM_v4.pdf</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>2025_11_16_ANOVA_one_way_Numero_de_chamada_Nivel_producao_3grupos.pdf</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>2025_11_20_tipoIES_IGC_contingencia.pdf</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>2025_12_09_participacao_PIBIC-EM_categoria_adm_corrigida_v4.omv.pdf</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>2025_12_09_Teste_X_quadrado_tipo_ies_corrigido_X_igc_categoria.pdf</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>2025_12_15_Teste_X_quadrado_categoria_adm_corrigida_X_igc_categoria.pdf</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>2025_12_09_Teste_X_quadrado_categoria_adm_corrigida_X_Regiao_corrigida.pdf</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>2025_12_13_Teste_X_quadrado_regiao_corrigida_X_igc_categoria.pdf</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>2025_11_16_grande_area_de_conhecimento_CAPES_participacao_PIBIC-EM.pdf</t>
+  </si>
+  <si>
+    <t>2025_11_16_ANOVA_grande_area_de_conhecimento_CAPES_participacao_PIBIC-EM.pdf</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>2025_11_16_Kruskal_Vallis_no_parametric_ANOVA_Numero_de_chamada_Nivel_producao_3grupos.pdf</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>2025_11_14_ANOVA_one_way_Numero_de_chamada_tipo_de_Instituicao.pdf</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Planejamento e gestão estratégica- o caso do CNPq.pdf</t>
   </si>
 </sst>
 </file>
@@ -1357,12 +1667,12 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF1F1F1F"/>
-      <name val="&quot;Google Sans Text&quot;"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
     <font>
-      <color rgb="FF444746"/>
-      <name val="&quot;Google Sans Text&quot;"/>
+      <color theme="1"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="6">
@@ -1486,7 +1796,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="44">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1574,6 +1884,9 @@
     <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="4" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
@@ -1594,10 +1907,25 @@
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="17" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf quotePrefix="1" borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf quotePrefix="1" borderId="0" fillId="0" fontId="18" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1620,6 +1948,10 @@
 </file>
 
 <file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -10111,11 +10443,58 @@
         <v>46006.0</v>
       </c>
     </row>
-    <row r="32" ht="15.75" customHeight="1"/>
-    <row r="33" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="16"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="16"/>
+      <c r="F32" s="16"/>
+      <c r="G32" s="16"/>
+      <c r="H32" s="16"/>
+      <c r="I32" s="16"/>
+      <c r="J32" s="16"/>
+      <c r="K32" s="16"/>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="A33" s="26">
+        <v>45698.0</v>
+      </c>
+      <c r="B33" s="26"/>
+      <c r="C33" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>260</v>
+      </c>
+      <c r="E33" s="16"/>
+      <c r="F33" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="G33" s="16"/>
+      <c r="H33" s="16"/>
+      <c r="I33" s="14" t="s">
+        <v>262</v>
+      </c>
+      <c r="J33" s="19" t="s">
+        <v>263</v>
+      </c>
+      <c r="K33" s="16"/>
+    </row>
     <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
-    <row r="36" ht="15.75" customHeight="1"/>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="A36" s="29"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="29"/>
+      <c r="H36" s="29"/>
+      <c r="I36" s="29"/>
+      <c r="J36" s="29"/>
+    </row>
     <row r="37" ht="15.75" customHeight="1"/>
     <row r="38" ht="15.75" customHeight="1"/>
     <row r="39" ht="15.75" customHeight="1"/>
@@ -10123,14 +10502,14 @@
     <row r="41" ht="15.75" customHeight="1"/>
     <row r="42" ht="15.75" customHeight="1"/>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="D43" s="29"/>
-      <c r="E43" s="29"/>
-      <c r="F43" s="29"/>
-      <c r="G43" s="29"/>
-      <c r="H43" s="29"/>
-      <c r="I43" s="29"/>
-      <c r="J43" s="29"/>
-      <c r="K43" s="29"/>
+      <c r="D43" s="30"/>
+      <c r="E43" s="30"/>
+      <c r="F43" s="30"/>
+      <c r="G43" s="30"/>
+      <c r="H43" s="30"/>
+      <c r="I43" s="30"/>
+      <c r="J43" s="30"/>
+      <c r="K43" s="30"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="D44" s="16"/>
@@ -10330,24 +10709,24 @@
     <row r="77" ht="15.75" customHeight="1"/>
     <row r="78" ht="15.75" customHeight="1"/>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="30"/>
+      <c r="A79" s="31"/>
       <c r="B79" s="25"/>
       <c r="C79" s="25"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="31" t="s">
-        <v>259</v>
+      <c r="A80" s="32" t="s">
+        <v>264</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="C80" s="19" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="14" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="B81" s="16"/>
       <c r="C81" s="16"/>
@@ -11315,12 +11694,13 @@
     <hyperlink r:id="rId53" ref="J30"/>
     <hyperlink r:id="rId54" ref="B31"/>
     <hyperlink r:id="rId55" ref="J31"/>
-    <hyperlink r:id="rId56" ref="C80"/>
+    <hyperlink r:id="rId56" ref="J33"/>
+    <hyperlink r:id="rId57" ref="C80"/>
   </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId57"/>
+  <drawing r:id="rId58"/>
 </worksheet>
 </file>
 
@@ -11344,39 +11724,39 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="32" t="s">
+      <c r="A1" s="33" t="s">
         <v>50</v>
       </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32" t="s">
-        <v>263</v>
-      </c>
-      <c r="D1" s="32" t="s">
-        <v>264</v>
-      </c>
-      <c r="E1" s="32" t="s">
-        <v>265</v>
-      </c>
-      <c r="F1" s="32" t="s">
-        <v>266</v>
-      </c>
-      <c r="G1" s="32" t="s">
-        <v>267</v>
-      </c>
-      <c r="H1" s="32" t="s">
+      <c r="B1" s="33"/>
+      <c r="C1" s="33" t="s">
         <v>268</v>
       </c>
-      <c r="I1" s="32" t="s">
+      <c r="D1" s="33" t="s">
         <v>269</v>
       </c>
-      <c r="J1" s="32" t="s">
+      <c r="E1" s="33" t="s">
         <v>270</v>
       </c>
-      <c r="K1" s="32" t="s">
+      <c r="F1" s="33" t="s">
         <v>271</v>
       </c>
-      <c r="L1" s="32" t="s">
+      <c r="G1" s="33" t="s">
         <v>272</v>
+      </c>
+      <c r="H1" s="33" t="s">
+        <v>273</v>
+      </c>
+      <c r="I1" s="33" t="s">
+        <v>274</v>
+      </c>
+      <c r="J1" s="33" t="s">
+        <v>275</v>
+      </c>
+      <c r="K1" s="33" t="s">
+        <v>276</v>
+      </c>
+      <c r="L1" s="33" t="s">
+        <v>277</v>
       </c>
       <c r="M1" s="16"/>
     </row>
@@ -11384,15 +11764,15 @@
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25" t="s">
-        <v>273</v>
-      </c>
-      <c r="M2" s="32"/>
+        <v>278</v>
+      </c>
+      <c r="M2" s="33"/>
     </row>
     <row r="3">
-      <c r="A3" s="33"/>
-      <c r="B3" s="33"/>
-      <c r="C3" s="33" t="s">
-        <v>274</v>
+      <c r="A3" s="34"/>
+      <c r="B3" s="34"/>
+      <c r="C3" s="34" t="s">
+        <v>279</v>
       </c>
     </row>
     <row r="4">
@@ -11400,47 +11780,47 @@
         <v>46007.0</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="33"/>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33" t="s">
-        <v>287</v>
+      <c r="A5" s="34"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="6">
@@ -11448,47 +11828,47 @@
         <v>46007.0</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="H6" s="14" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="K6" s="14" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="L6" s="14" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="M6" s="19" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="33"/>
-      <c r="B7" s="33"/>
-      <c r="C7" s="33" t="s">
-        <v>298</v>
+      <c r="A7" s="34"/>
+      <c r="B7" s="34"/>
+      <c r="C7" s="34" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="8">
@@ -11496,45 +11876,45 @@
         <v>46007.0</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="M8" s="19" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="s">
-        <v>308</v>
+      <c r="A9" s="34" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="10">
@@ -11542,40 +11922,45 @@
         <v>46007.0</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="M10" s="19" t="s">
-        <v>317</v>
+        <v>322</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21">
+        <v>45698.0</v>
       </c>
     </row>
   </sheetData>
@@ -11607,155 +11992,568 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="32.43"/>
-    <col customWidth="1" min="2" max="2" width="41.43"/>
-    <col customWidth="1" min="3" max="3" width="60.57"/>
-    <col customWidth="1" min="4" max="4" width="74.43"/>
-    <col customWidth="1" min="5" max="5" width="56.71"/>
+    <col customWidth="1" min="1" max="1" width="24.14"/>
+    <col customWidth="1" min="2" max="2" width="40.57"/>
+    <col customWidth="1" min="3" max="3" width="44.43"/>
+    <col customWidth="1" min="4" max="4" width="38.57"/>
+    <col customWidth="1" min="5" max="5" width="30.71"/>
+    <col customWidth="1" min="6" max="6" width="42.71"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="34" t="s">
-        <v>318</v>
-      </c>
-      <c r="E1" s="35"/>
+      <c r="A1" s="35"/>
+      <c r="E1" s="36"/>
     </row>
     <row r="2">
-      <c r="A2" s="35" t="s">
-        <v>319</v>
-      </c>
-      <c r="B2" s="35" t="s">
-        <v>320</v>
-      </c>
-      <c r="C2" s="35" t="s">
-        <v>321</v>
-      </c>
-      <c r="D2" s="35" t="s">
-        <v>322</v>
-      </c>
-      <c r="E2" s="35"/>
+      <c r="A2" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="37" t="s">
+        <v>323</v>
+      </c>
+      <c r="C2" s="37" t="s">
+        <v>324</v>
+      </c>
+      <c r="D2" s="37" t="s">
+        <v>325</v>
+      </c>
+      <c r="E2" s="37" t="s">
+        <v>326</v>
+      </c>
+      <c r="F2" s="38" t="s">
+        <v>327</v>
+      </c>
+      <c r="G2" s="38" t="s">
+        <v>328</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="36" t="s">
-        <v>323</v>
-      </c>
-      <c r="B3" s="37" t="s">
-        <v>324</v>
-      </c>
-      <c r="C3" s="36" t="s">
-        <v>325</v>
-      </c>
-      <c r="D3" s="36" t="s">
-        <v>326</v>
-      </c>
-      <c r="E3" s="35"/>
+      <c r="A3" s="39" t="s">
+        <v>329</v>
+      </c>
+      <c r="B3" s="39" t="s">
+        <v>330</v>
+      </c>
+      <c r="C3" s="39" t="s">
+        <v>331</v>
+      </c>
+      <c r="D3" s="39" t="s">
+        <v>332</v>
+      </c>
+      <c r="E3" s="39" t="s">
+        <v>333</v>
+      </c>
+      <c r="F3" s="40" t="s">
+        <v>334</v>
+      </c>
+      <c r="G3" s="41" t="s">
+        <v>335</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="36" t="s">
-        <v>327</v>
-      </c>
-      <c r="B4" s="37" t="s">
-        <v>328</v>
-      </c>
-      <c r="C4" s="36" t="s">
-        <v>329</v>
-      </c>
-      <c r="D4" s="35" t="s">
-        <v>330</v>
-      </c>
-      <c r="E4" s="35"/>
+      <c r="A4" s="39" t="s">
+        <v>336</v>
+      </c>
+      <c r="B4" s="39" t="s">
+        <v>337</v>
+      </c>
+      <c r="C4" s="39" t="s">
+        <v>338</v>
+      </c>
+      <c r="D4" s="39" t="s">
+        <v>332</v>
+      </c>
+      <c r="E4" s="39" t="s">
+        <v>339</v>
+      </c>
+      <c r="F4" s="40" t="s">
+        <v>340</v>
+      </c>
+      <c r="G4" s="41" t="s">
+        <v>341</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="36" t="s">
-        <v>331</v>
-      </c>
-      <c r="B5" s="37" t="s">
+      <c r="A5" s="39" t="s">
+        <v>342</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>343</v>
+      </c>
+      <c r="C5" s="39" t="s">
+        <v>344</v>
+      </c>
+      <c r="D5" s="39" t="s">
         <v>332</v>
       </c>
-      <c r="C5" s="36" t="s">
-        <v>333</v>
-      </c>
-      <c r="D5" s="36" t="s">
-        <v>334</v>
-      </c>
-      <c r="E5" s="35"/>
+      <c r="E5" s="39" t="s">
+        <v>345</v>
+      </c>
+      <c r="F5" s="40" t="s">
+        <v>346</v>
+      </c>
+      <c r="G5" s="41" t="s">
+        <v>347</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="s">
-        <v>335</v>
-      </c>
-      <c r="B6" s="37" t="s">
-        <v>336</v>
-      </c>
-      <c r="C6" s="36" t="s">
-        <v>337</v>
-      </c>
-      <c r="D6" s="35" t="s">
-        <v>338</v>
-      </c>
-      <c r="E6" s="35"/>
+      <c r="A6" s="39" t="s">
+        <v>348</v>
+      </c>
+      <c r="B6" s="39" t="s">
+        <v>349</v>
+      </c>
+      <c r="C6" s="39" t="s">
+        <v>350</v>
+      </c>
+      <c r="D6" s="39" t="s">
+        <v>351</v>
+      </c>
+      <c r="E6" s="39" t="s">
+        <v>352</v>
+      </c>
+      <c r="F6" s="40" t="s">
+        <v>353</v>
+      </c>
+      <c r="G6" s="40" t="s">
+        <v>354</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="36"/>
-      <c r="B7" s="35"/>
-      <c r="C7" s="35"/>
-      <c r="D7" s="36"/>
-      <c r="E7" s="35"/>
+      <c r="A7" s="39" t="s">
+        <v>355</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>356</v>
+      </c>
+      <c r="C7" s="39" t="s">
+        <v>357</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>351</v>
+      </c>
+      <c r="E7" s="39" t="s">
+        <v>358</v>
+      </c>
+      <c r="F7" s="40" t="s">
+        <v>359</v>
+      </c>
+      <c r="G7" s="41" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="40" t="s">
+        <v>361</v>
+      </c>
+      <c r="B8" s="40" t="s">
+        <v>362</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>363</v>
+      </c>
+      <c r="D8" s="40" t="s">
+        <v>364</v>
+      </c>
+      <c r="E8" s="40" t="s">
+        <v>365</v>
+      </c>
+      <c r="F8" s="40" t="s">
+        <v>366</v>
+      </c>
+      <c r="G8" s="40" t="s">
+        <v>367</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="17" t="s">
-        <v>339</v>
+      <c r="A9" s="40" t="s">
+        <v>368</v>
+      </c>
+      <c r="B9" s="40" t="s">
+        <v>369</v>
+      </c>
+      <c r="C9" s="40" t="s">
+        <v>370</v>
+      </c>
+      <c r="D9" s="40" t="s">
+        <v>371</v>
+      </c>
+      <c r="E9" s="40" t="s">
+        <v>372</v>
+      </c>
+      <c r="F9" s="40" t="s">
+        <v>373</v>
+      </c>
+      <c r="G9" s="41" t="s">
+        <v>374</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="35" t="s">
-        <v>340</v>
-      </c>
-      <c r="B10" s="35" t="s">
-        <v>341</v>
-      </c>
-      <c r="C10" s="35" t="s">
-        <v>342</v>
+      <c r="A10" s="39" t="s">
+        <v>375</v>
+      </c>
+      <c r="B10" s="39" t="s">
+        <v>376</v>
+      </c>
+      <c r="C10" s="39" t="s">
+        <v>377</v>
+      </c>
+      <c r="D10" s="40" t="s">
+        <v>378</v>
+      </c>
+      <c r="E10" s="40" t="s">
+        <v>379</v>
+      </c>
+      <c r="F10" s="40" t="s">
+        <v>380</v>
+      </c>
+      <c r="G10" s="40" t="s">
+        <v>381</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="36" t="s">
-        <v>343</v>
-      </c>
-      <c r="B11" s="36" t="s">
-        <v>344</v>
-      </c>
-      <c r="C11" s="35" t="s">
-        <v>345</v>
+      <c r="A11" s="39" t="s">
+        <v>368</v>
+      </c>
+      <c r="B11" s="39" t="s">
+        <v>382</v>
+      </c>
+      <c r="C11" s="39" t="s">
+        <v>383</v>
+      </c>
+      <c r="D11" s="40" t="s">
+        <v>384</v>
+      </c>
+      <c r="E11" s="40" t="s">
+        <v>385</v>
+      </c>
+      <c r="F11" s="40" t="s">
+        <v>386</v>
+      </c>
+      <c r="G11" s="41" t="s">
+        <v>387</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="s">
-        <v>346</v>
-      </c>
-      <c r="B12" s="36" t="s">
-        <v>347</v>
-      </c>
-      <c r="C12" s="35" t="s">
-        <v>348</v>
+      <c r="A12" s="39" t="s">
+        <v>388</v>
+      </c>
+      <c r="B12" s="39" t="s">
+        <v>389</v>
+      </c>
+      <c r="C12" s="39" t="s">
+        <v>390</v>
+      </c>
+      <c r="D12" s="40" t="s">
+        <v>391</v>
+      </c>
+      <c r="E12" s="40" t="s">
+        <v>392</v>
+      </c>
+      <c r="F12" s="40" t="s">
+        <v>393</v>
+      </c>
+      <c r="G12" s="41" t="s">
+        <v>394</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="36" t="s">
-        <v>349</v>
-      </c>
-      <c r="B13" s="36" t="s">
-        <v>350</v>
-      </c>
-      <c r="C13" s="36" t="s">
-        <v>351</v>
+      <c r="A13" s="39" t="s">
+        <v>395</v>
+      </c>
+      <c r="B13" s="39" t="s">
+        <v>396</v>
+      </c>
+      <c r="C13" s="39" t="s">
+        <v>397</v>
+      </c>
+      <c r="D13" s="40" t="s">
+        <v>332</v>
+      </c>
+      <c r="E13" s="40" t="s">
+        <v>398</v>
+      </c>
+      <c r="F13" s="40" t="s">
+        <v>399</v>
+      </c>
+      <c r="G13" s="41" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="40" t="s">
+        <v>401</v>
+      </c>
+      <c r="B14" s="40" t="s">
+        <v>402</v>
+      </c>
+      <c r="C14" s="40" t="s">
+        <v>403</v>
+      </c>
+      <c r="D14" s="40" t="s">
+        <v>332</v>
+      </c>
+      <c r="E14" s="40" t="s">
+        <v>404</v>
+      </c>
+      <c r="F14" s="40" t="s">
+        <v>405</v>
+      </c>
+      <c r="G14" s="41" t="s">
+        <v>406</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:C9"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="6.29"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="42" t="s">
+        <v>407</v>
+      </c>
+      <c r="B1" s="42" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="43" t="s">
+        <v>409</v>
+      </c>
+      <c r="B2" s="42" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="43" t="s">
+        <v>411</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="43" t="s">
+        <v>413</v>
+      </c>
+      <c r="B4" s="42" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="43" t="s">
+        <v>415</v>
+      </c>
+      <c r="B5" s="42" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="43" t="s">
+        <v>417</v>
+      </c>
+      <c r="B6" s="42" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="43" t="s">
+        <v>419</v>
+      </c>
+      <c r="B7" s="42" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="43" t="s">
+        <v>400</v>
+      </c>
+      <c r="B8" s="42" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="43" t="s">
+        <v>422</v>
+      </c>
+      <c r="B9" s="42" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="43" t="s">
+        <v>424</v>
+      </c>
+      <c r="B10" s="42" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="43" t="s">
+        <v>426</v>
+      </c>
+      <c r="B11" s="42" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="43" t="s">
+        <v>427</v>
+      </c>
+      <c r="B12" s="42" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="43" t="s">
+        <v>429</v>
+      </c>
+      <c r="B13" s="42" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="43" t="s">
+        <v>431</v>
+      </c>
+      <c r="B14" s="42" t="s">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="43" t="s">
+        <v>432</v>
+      </c>
+      <c r="B15" s="42" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="43" t="s">
+        <v>434</v>
+      </c>
+      <c r="B16" s="42" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="43" t="s">
+        <v>436</v>
+      </c>
+      <c r="B17" s="42" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="43" t="s">
+        <v>438</v>
+      </c>
+      <c r="B18" s="42" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="43" t="s">
+        <v>440</v>
+      </c>
+      <c r="B19" s="42" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="43" t="s">
+        <v>394</v>
+      </c>
+      <c r="B20" s="42" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="43" t="s">
+        <v>443</v>
+      </c>
+      <c r="B21" s="42" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="43" t="s">
+        <v>444</v>
+      </c>
+      <c r="B22" s="42" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="43" t="s">
+        <v>445</v>
+      </c>
+      <c r="B23" s="42" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="43" t="s">
+        <v>447</v>
+      </c>
+      <c r="B24" s="42" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="43" t="s">
+        <v>449</v>
+      </c>
+      <c r="B25" s="42" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="43" t="s">
+        <v>450</v>
+      </c>
+      <c r="B26" s="42" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="43" t="s">
+        <v>451</v>
+      </c>
+      <c r="B27" s="42" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="43" t="s">
+        <v>452</v>
+      </c>
+      <c r="B28" s="42" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="43" t="s">
+        <v>453</v>
+      </c>
+      <c r="B29" s="42" t="s">
+        <v>454</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Modelo Mulivariado IF/CEFEs e Universidades Federais
Acréscimo do modelo Quasi-Poisson Universidades Federais e IFs/CEFETs.
</commit_message>
<xml_diff>
--- a/06_Roteiros_Estatis/Acompanhamento_Analises_PIBICEM.xlsx
+++ b/06_Roteiros_Estatis/Acompanhamento_Analises_PIBICEM.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="544" uniqueCount="455">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="457">
   <si>
     <t>Nível de análise</t>
   </si>
@@ -950,6 +950,12 @@
   </si>
   <si>
     <t>2026_02_10_modelo_multivariado_3_.pdf</t>
+  </si>
+  <si>
+    <t>Avaliar o efeito da participação no PIBIC-EM entre pesquisadores dos IF/CEFETs e das Universidades Federais</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os resultados deste modelo específico (tabela \ref{tab:poisson-federal}) corroboram a tendência observada: mantendo constante a produtividade acadêmica, os docentes dos Institutos Federais apresentam uma probabilidade de participação 15% superior à de seus pares nas Universidades Federais ($IRR=1{,}15$; $IC~95\%: 1{,}01\text{--}1{,}31$; $p=0{,}033$). </t>
   </si>
   <si>
     <t>Quais instituições retornam sistematicamente ao programa?</t>
@@ -9259,7 +9265,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="5.29"/>
+    <col customWidth="1" min="1" max="1" width="20.0"/>
     <col customWidth="1" min="2" max="2" width="27.29"/>
     <col customWidth="1" min="3" max="3" width="26.0"/>
     <col customWidth="1" min="4" max="4" width="29.14"/>
@@ -10457,9 +10463,6 @@
       <c r="K32" s="16"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="26">
-        <v>45698.0</v>
-      </c>
       <c r="B33" s="26"/>
       <c r="C33" s="14" t="s">
         <v>259</v>
@@ -10479,9 +10482,32 @@
       <c r="J33" s="19" t="s">
         <v>263</v>
       </c>
-      <c r="K33" s="16"/>
-    </row>
-    <row r="34" ht="15.75" customHeight="1"/>
+      <c r="K33" s="26">
+        <v>45698.0</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="B34" s="16"/>
+      <c r="C34" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="D34" s="14" t="s">
+        <v>264</v>
+      </c>
+      <c r="E34" s="16"/>
+      <c r="F34" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="G34" s="16"/>
+      <c r="H34" s="16"/>
+      <c r="I34" s="14" t="s">
+        <v>265</v>
+      </c>
+      <c r="J34" s="16"/>
+      <c r="K34" s="26">
+        <v>45700.0</v>
+      </c>
+    </row>
     <row r="35" ht="15.75" customHeight="1"/>
     <row r="36" ht="15.75" customHeight="1">
       <c r="A36" s="29"/>
@@ -10715,18 +10741,18 @@
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="A80" s="32" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B80" s="14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C80" s="19" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="A81" s="14" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B81" s="16"/>
       <c r="C81" s="16"/>
@@ -11729,34 +11755,34 @@
       </c>
       <c r="B1" s="33"/>
       <c r="C1" s="33" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D1" s="33" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E1" s="33" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="F1" s="33" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="G1" s="33" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="H1" s="33" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="I1" s="33" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="J1" s="33" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="K1" s="33" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="L1" s="33" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="M1" s="16"/>
     </row>
@@ -11764,7 +11790,7 @@
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="M2" s="33"/>
     </row>
@@ -11772,7 +11798,7 @@
       <c r="A3" s="34"/>
       <c r="B3" s="34"/>
       <c r="C3" s="34" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4">
@@ -11780,47 +11806,47 @@
         <v>46007.0</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D4" s="14" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="E4" s="14" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F4" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="H4" s="14" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="I4" s="14" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="J4" s="14" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="K4" s="14" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="L4" s="14" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="M4" s="19" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="34"/>
       <c r="B5" s="34"/>
       <c r="C5" s="34" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
     </row>
     <row r="6">
@@ -11828,47 +11854,47 @@
         <v>46007.0</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="E6" s="14" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F6" s="14" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="H6" s="14" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I6" s="14" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="J6" s="14" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="K6" s="14" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="L6" s="14" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="M6" s="19" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="34"/>
       <c r="B7" s="34"/>
       <c r="C7" s="34" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
     </row>
     <row r="8">
@@ -11876,45 +11902,45 @@
         <v>46007.0</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="E8" s="14" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F8" s="14" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G8" s="14" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="J8" s="14" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="K8" s="14" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="L8" s="14" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="M8" s="19" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="34" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
     </row>
     <row r="10">
@@ -11922,40 +11948,40 @@
         <v>46007.0</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D10" s="14" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="E10" s="14" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F10" s="14" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="G10" s="14" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="I10" s="14" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="J10" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="K10" s="14" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="L10" s="14" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="M10" s="19" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
     </row>
     <row r="12">
@@ -12009,298 +12035,298 @@
         <v>42</v>
       </c>
       <c r="B2" s="37" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="C2" s="37" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D2" s="37" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E2" s="37" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F2" s="38" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="G2" s="38" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="39" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B3" s="39" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C3" s="39" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D3" s="39" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E3" s="39" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F3" s="40" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="G3" s="41" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="39" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B4" s="39" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C4" s="39" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D4" s="39" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E4" s="39" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="F4" s="40" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="G4" s="41" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="39" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C5" s="39" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D5" s="39" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E5" s="39" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="F5" s="40" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="G5" s="41" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="39" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B6" s="39" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C6" s="39" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D6" s="39" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E6" s="39" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="F6" s="40" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="G6" s="40" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="39" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B7" s="39" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="C7" s="39" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="D7" s="39" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E7" s="39" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="F7" s="40" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="G7" s="41" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="40" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B8" s="40" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D8" s="40" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E8" s="40" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="F8" s="40" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="G8" s="40" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="40" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B9" s="40" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="C9" s="40" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D9" s="40" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E9" s="40" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F9" s="40" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="G9" s="41" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="39" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C10" s="39" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D10" s="40" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E10" s="40" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F10" s="40" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="G10" s="40" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="39" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C11" s="39" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="D11" s="40" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E11" s="40" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F11" s="40" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="G11" s="41" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="39" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="C12" s="39" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D12" s="40" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E12" s="40" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F12" s="40" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="G12" s="41" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="39" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B13" s="39" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C13" s="39" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="F13" s="40" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="G13" s="41" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="40" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B14" s="40" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C14" s="40" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D14" s="40" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="E14" s="40" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="F14" s="40" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="G14" s="41" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>
@@ -12323,87 +12349,87 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="42" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B1" s="42" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="43" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B2" s="42" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="43" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B3" s="42" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="43" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="43" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B5" s="42" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="43" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B6" s="42" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="43" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B7" s="42" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="43" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B8" s="42" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="43" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B9" s="42" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="43" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B10" s="42" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="43" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B11" s="42" t="s">
         <v>58</v>
@@ -12411,119 +12437,119 @@
     </row>
     <row r="12">
       <c r="A12" s="43" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B12" s="42" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="43" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B13" s="42" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="43" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B14" s="42" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="43" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B15" s="42" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="43" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B16" s="42" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="43" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B17" s="42" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="43" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B18" s="42" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="43" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B19" s="42" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="43" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B20" s="42" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="43" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B21" s="42" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="43" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B22" s="42" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="43" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B23" s="42" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="43" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B24" s="42" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="43" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B25" s="42" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="43" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B26" s="42" t="s">
         <v>191</v>
@@ -12531,7 +12557,7 @@
     </row>
     <row r="27">
       <c r="A27" s="43" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B27" s="42" t="s">
         <v>184</v>
@@ -12539,7 +12565,7 @@
     </row>
     <row r="28">
       <c r="A28" s="43" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B28" s="42" t="s">
         <v>207</v>
@@ -12547,10 +12573,10 @@
     </row>
     <row r="29">
       <c r="A29" s="43" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B29" s="42" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
     </row>
   </sheetData>

</xml_diff>